<commit_message>
Destaca em amarelo os tópicos pedidos e adiciona aba Respostas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P7w24RHndLrBsJYLAj6Rs3
</commit_message>
<xml_diff>
--- a/pcp-gestao-estoques/Exercicio_Resolvido_Gestao_Estoques.xlsx
+++ b/pcp-gestao-estoques/Exercicio_Resolvido_Gestao_Estoques.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Parâmetros" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="1 - Qtde Fixa" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2 - Período Fixo" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Respostas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Parâmetros" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="1 - Qtde Fixa" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2 - Período Fixo" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -47,12 +48,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -76,13 +77,13 @@
   <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -455,6 +456,156 @@
   <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
+    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>RESPOSTAS DO EXERCÍCIO (nível de serviço 95%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Método 1 – Ponto de Pedido / Quantidade Fixa de Encomenda</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Ponto de Pedido</t>
+        </is>
+      </c>
+      <c r="B4" s="3">
+        <f>'1 - Qtde Fixa'!B33</f>
+        <v/>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>cocos</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Quantidade do Lote (Lote Econômico Q0)</t>
+        </is>
+      </c>
+      <c r="B5" s="3">
+        <f>'1 - Qtde Fixa'!B6</f>
+        <v/>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>cocos</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Estoque de Segurança</t>
+        </is>
+      </c>
+      <c r="B6" s="3">
+        <f>'1 - Qtde Fixa'!C33</f>
+        <v/>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>cocos</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Método 2 – Estoque Máximo / Período Fixo de Encomenda</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Estoque Máximo</t>
+        </is>
+      </c>
+      <c r="B9" s="3">
+        <f>'2 - Período Fixo'!B42</f>
+        <v/>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>cocos</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Período Fixo de Encomenda</t>
+        </is>
+      </c>
+      <c r="B10" s="3">
+        <f>'2 - Período Fixo'!B5</f>
+        <v/>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>dias</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Estoque de Segurança</t>
+        </is>
+      </c>
+      <c r="B11" s="3">
+        <f>'2 - Período Fixo'!C42</f>
+        <v/>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>cocos</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Método 1: sempre que o estoque (físico + a receber) chegar a 180, pedir 122 cocos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Método 2: a cada 2 dias, pedir 350 − saldo físico − compras a receber.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
@@ -473,7 +624,7 @@
           <t>Custo de frete por encomenda (Ce)</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="4" t="n">
         <v>15</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -488,7 +639,7 @@
           <t>Custo de manter 1 unidade por dia (I)</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="4" t="n">
         <v>0.15</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -503,7 +654,7 @@
           <t>Demanda média diária (D)</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="4" t="n">
         <v>75</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -518,7 +669,7 @@
           <t>Demanda máxima diária</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B6" s="4" t="n">
         <v>100</v>
       </c>
       <c r="C6" t="inlineStr">
@@ -533,7 +684,7 @@
           <t>Demanda mínima diária</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="4" t="n">
         <v>51</v>
       </c>
       <c r="C7" t="inlineStr">
@@ -548,7 +699,7 @@
           <t>Tempo médio de reposição (TR)</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="4" t="n">
         <v>1.7</v>
       </c>
       <c r="C8" t="inlineStr">
@@ -563,7 +714,7 @@
           <t>Tempo de reposição máximo</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C9" t="inlineStr">
@@ -578,7 +729,7 @@
           <t>Tempo de reposição mínimo</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C10" t="inlineStr">
@@ -593,7 +744,7 @@
           <t>Dias no mês</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B11" s="4" t="n">
         <v>30</v>
       </c>
       <c r="C11" t="inlineStr">
@@ -608,7 +759,7 @@
           <t>Nível de serviço desejado</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B12" s="5" t="n">
         <v>0.95</v>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -650,7 +801,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -679,7 +830,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>PASSO 1 – Lote Econômico (Q0)</t>
         </is>
@@ -698,18 +849,18 @@
           <t>Q0 calculado</t>
         </is>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="7">
         <f>SQRT(2*'Parâmetros'!B5*'Parâmetros'!B3/'Parâmetros'!B4)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Q0 adotado (arredondado)</t>
         </is>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="3">
         <f>ROUND(B5,0)</f>
         <v/>
       </c>
@@ -720,7 +871,7 @@
           <t>Custo mensal de armazenar estoque de ciclo = Q/2 × I × 30</t>
         </is>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="8">
         <f>B6/2*'Parâmetros'!B4*'Parâmetros'!B11</f>
         <v/>
       </c>
@@ -731,7 +882,7 @@
           <t>Custo mensal de encomendar = (D × 30 / Q) × Ce</t>
         </is>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="8">
         <f>'Parâmetros'!B5*'Parâmetros'!B11/B6*'Parâmetros'!B3</f>
         <v/>
       </c>
@@ -742,65 +893,65 @@
           <t>Custo mensal total</t>
         </is>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="8">
         <f>B7+B8</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>PASSO 2 – Distribuição da demanda no tempo de reposição (100 sorteios da aba Planilha1 do professor)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Classe de</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>até</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Frequência</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Prob. (%)</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>Freq. acum.</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Prob. acum. (%)</t>
         </is>
       </c>
-      <c r="G12" s="8" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>TR sorteado</t>
         </is>
       </c>
-      <c r="H12" s="8" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Demanda dia 1</t>
         </is>
       </c>
-      <c r="I12" s="8" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Demanda dia 2</t>
         </is>
       </c>
-      <c r="J12" s="8" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>Demanda no TR</t>
         </is>
@@ -1329,7 +1480,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>PASSO 3 – Ponto de Pedido e Estoque de Segurança</t>
         </is>
@@ -1367,22 +1518,22 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>Nível de serviço</t>
         </is>
       </c>
-      <c r="B31" s="8" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>Ponto de Pedido</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>Estoque de Segurança</t>
         </is>
       </c>
-      <c r="D31" s="8" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>Custo mensal do ES (R$)</t>
         </is>
@@ -1410,7 +1561,7 @@
         <f>B32-$B$30</f>
         <v/>
       </c>
-      <c r="D32" s="5">
+      <c r="D32" s="7">
         <f>C32*'Parâmetros'!$B$4*'Parâmetros'!$B$11</f>
         <v/>
       </c>
@@ -1429,11 +1580,11 @@
       <c r="A33" s="11" t="n">
         <v>0.95</v>
       </c>
-      <c r="B33" s="6">
+      <c r="B33" s="3">
         <f>INDEX($B$13:$B$27,MATCH(TRUE,INDEX($F$13:$F$27&gt;=0.95-1E-9,0),0))</f>
         <v/>
       </c>
-      <c r="C33" s="6">
+      <c r="C33" s="3">
         <f>B33-$B$30</f>
         <v/>
       </c>
@@ -1464,7 +1615,7 @@
         <f>B34-$B$30</f>
         <v/>
       </c>
-      <c r="D34" s="5">
+      <c r="D34" s="7">
         <f>C34*'Parâmetros'!$B$4*'Parâmetros'!$B$11</f>
         <v/>
       </c>
@@ -1492,7 +1643,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>RESPOSTA: pedir 122 cocos sempre que o estoque providenciado (físico + a receber) chegar a 180 cocos (ES = 52,5).</t>
         </is>
@@ -2578,7 +2729,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2610,7 +2761,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>PASSO 1 – Período ótimo de encomenda</t>
         </is>
@@ -2622,24 +2773,24 @@
           <t>T = Q0 / Demanda média diária</t>
         </is>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="7">
         <f>'1 - Qtde Fixa'!B5/'Parâmetros'!B5</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>T adotado (dias inteiros)</t>
         </is>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="3">
         <f>ROUND(B4,0)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>PASSO 2 – Tempo de cobertura = T + TR</t>
         </is>
@@ -2690,74 +2841,74 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>PASSO 3 – Demanda no tempo de cobertura (100 sorteios: TR 1 dia 30% / 2 dias 70%; demanda diária de 51 a 100)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Classe de</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>até</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Frequência</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Prob. (%)</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Freq. acum.</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Prob. acum. (%)</t>
         </is>
       </c>
-      <c r="H14" s="8" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>TR sorteado</t>
         </is>
       </c>
-      <c r="I14" s="8" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>Dia 1</t>
         </is>
       </c>
-      <c r="J14" s="8" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>Dia 2</t>
         </is>
       </c>
-      <c r="K14" s="8" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>Dia 3</t>
         </is>
       </c>
-      <c r="L14" s="8" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>Dia 4</t>
         </is>
       </c>
-      <c r="M14" s="8" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>Cobertura (dias)</t>
         </is>
       </c>
-      <c r="N14" s="8" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>Demanda na cobertura</t>
         </is>
@@ -3852,7 +4003,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>PASSO 4 – Estoque Máximo e Estoque de Segurança</t>
         </is>
@@ -3882,22 +4033,22 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>Nível de serviço</t>
         </is>
       </c>
-      <c r="B40" s="8" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Estoque Máximo</t>
         </is>
       </c>
-      <c r="C40" s="8" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>Estoque de Segurança</t>
         </is>
       </c>
-      <c r="D40" s="8" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>Custo mensal do ES (R$)</t>
         </is>
@@ -3935,7 +4086,7 @@
         <f>B41-$B$11</f>
         <v/>
       </c>
-      <c r="D41" s="5">
+      <c r="D41" s="7">
         <f>C41*'Parâmetros'!$B$4*'Parâmetros'!$B$11</f>
         <v/>
       </c>
@@ -3967,11 +4118,11 @@
       <c r="A42" s="11" t="n">
         <v>0.95</v>
       </c>
-      <c r="B42" s="6">
+      <c r="B42" s="3">
         <f>INDEX($B$15:$B$37,MATCH(TRUE,INDEX($F$15:$F$37&gt;=0.95-1E-9,0),0))</f>
         <v/>
       </c>
-      <c r="C42" s="6">
+      <c r="C42" s="3">
         <f>B42-$B$11</f>
         <v/>
       </c>
@@ -4012,7 +4163,7 @@
         <f>B43-$B$11</f>
         <v/>
       </c>
-      <c r="D43" s="5">
+      <c r="D43" s="7">
         <f>C43*'Parâmetros'!$B$4*'Parâmetros'!$B$11</f>
         <v/>
       </c>
@@ -4063,7 +4214,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>RESPOSTA: a cada 2 dias, encomendar (350 − saldo físico − compras a receber) cocos (ES = 72,5).</t>
         </is>

</xml_diff>